<commit_message>
minor edit to spreadsheet
</commit_message>
<xml_diff>
--- a/ft4232h-bob-v0/PartsOrder-FT232H-v0.xlsx
+++ b/ft4232h-bob-v0/PartsOrder-FT232H-v0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mwg/code/EE Projects 2022-/ComputerBreakout/Design/FT4232H Breakout/ft4232h-bob-v0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307036D6-1CA2-3740-A471-86C72F46826B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2032A8-E282-7C43-91B7-6323CE18A42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="680" windowWidth="26480" windowHeight="17420" xr2:uid="{7C62EEA5-59C9-AF4A-87E9-63E817F36AD7}"/>
+    <workbookView xWindow="900" yWindow="880" windowWidth="26480" windowHeight="17420" xr2:uid="{7C62EEA5-59C9-AF4A-87E9-63E817F36AD7}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="190">
   <si>
     <t>Desc</t>
   </si>
@@ -604,6 +604,9 @@
   </si>
   <si>
     <t>R3,R7,R9,R10,R11-14</t>
+  </si>
+  <si>
+    <t>FT4232H Breakout Board</t>
   </si>
 </sst>
 </file>
@@ -757,7 +760,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -806,21 +809,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -832,10 +825,7 @@
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -1156,12 +1146,12 @@
   <dimension ref="A1:Q50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="45.5" style="32" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="32" customWidth="1"/>
+    <col min="1" max="1" width="45.5" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
     <col min="3" max="3" width="1.6640625" customWidth="1"/>
     <col min="4" max="4" width="6.33203125" customWidth="1"/>
     <col min="5" max="5" width="6" customWidth="1"/>
-    <col min="6" max="6" width="5.83203125" style="36" customWidth="1"/>
+    <col min="6" max="6" width="5.83203125" style="31" customWidth="1"/>
     <col min="9" max="10" width="33.6640625" customWidth="1"/>
     <col min="11" max="11" width="19.33203125" customWidth="1"/>
     <col min="12" max="12" width="48.5" customWidth="1"/>
@@ -1174,10 +1164,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="13" customFormat="1" ht="34" x14ac:dyDescent="0.2">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="B1" s="13" t="s">
         <v>8</v>
       </c>
       <c r="D1" s="13" t="s">
@@ -1186,7 +1176,7 @@
       <c r="E1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="30" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="13" t="s">
@@ -1246,11 +1236,11 @@
         <v/>
       </c>
       <c r="O3" t="str">
-        <f>IF(ISNUMBER(SEARCH(O$1,$I3)),1,"")</f>
+        <f t="shared" ref="O3:P5" si="1">IF(ISNUMBER(SEARCH(O$1,$I3)),1,"")</f>
         <v/>
       </c>
       <c r="P3" t="str">
-        <f>IF(ISNUMBER(SEARCH(P$1,$I3)),1,"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q3" t="str">
@@ -1260,7 +1250,7 @@
     </row>
     <row r="4" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>38</v>
+        <v>189</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="1"/>
@@ -1269,11 +1259,11 @@
         <v/>
       </c>
       <c r="O4" t="str">
-        <f>IF(ISNUMBER(SEARCH(O$1,$I4)),1,"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="P4" t="str">
-        <f>IF(ISNUMBER(SEARCH(P$1,$I4)),1,"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q4" t="str">
@@ -1282,10 +1272,10 @@
       </c>
     </row>
     <row r="5" spans="1:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="37">
+      <c r="B5" s="8">
         <v>3</v>
       </c>
       <c r="G5" s="3"/>
@@ -1295,11 +1285,11 @@
         <v/>
       </c>
       <c r="O5" t="str">
-        <f>IF(ISNUMBER(SEARCH(O$1,$I5)),1,"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="P5" t="str">
-        <f>IF(ISNUMBER(SEARCH(P$1,$I5)),1,"")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="Q5" t="str">
@@ -1308,24 +1298,24 @@
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A6" s="30" t="s">
+      <c r="A6" t="s">
         <v>144</v>
       </c>
-      <c r="B6" s="38" t="s">
+      <c r="B6" s="32" t="s">
         <v>9</v>
       </c>
       <c r="D6">
         <v>1</v>
       </c>
       <c r="E6">
-        <f t="shared" ref="E6:E20" si="1">ROUNDUP(D6*$B$5,0)</f>
+        <f t="shared" ref="E6:E20" si="2">ROUNDUP(D6*$B$5,0)</f>
         <v>3</v>
       </c>
-      <c r="F6" s="36">
+      <c r="F6" s="31">
         <v>6.35</v>
       </c>
       <c r="G6" s="3">
-        <f t="shared" ref="G6:G8" si="2">E6*F6</f>
+        <f t="shared" ref="G6:G8" si="3">E6*F6</f>
         <v>19.049999999999997</v>
       </c>
       <c r="H6" s="1" t="s">
@@ -1342,24 +1332,24 @@
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A7" s="34" t="s">
+      <c r="A7" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="38" t="s">
+      <c r="B7" s="32" t="s">
         <v>145</v>
       </c>
       <c r="D7">
         <v>1</v>
       </c>
       <c r="E7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F7" s="36">
+      <c r="F7" s="31">
         <v>1.1599999999999999</v>
       </c>
       <c r="G7" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.4799999999999995</v>
       </c>
       <c r="H7" s="1" t="s">
@@ -1376,24 +1366,24 @@
       </c>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A8" s="34" t="s">
+      <c r="A8" t="s">
         <v>136</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="32" t="s">
         <v>42</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F8" s="36">
+      <c r="F8" s="31">
         <v>2.5000000000000001E-2</v>
       </c>
       <c r="G8" s="3">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7.5000000000000011E-2</v>
       </c>
       <c r="H8" s="1" t="s">
@@ -1410,24 +1400,24 @@
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A9" s="34" t="s">
+      <c r="A9" t="s">
         <v>130</v>
       </c>
-      <c r="B9" s="38" t="s">
+      <c r="B9" s="32" t="s">
         <v>148</v>
       </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="31">
         <v>1.3299999999999999E-2</v>
       </c>
       <c r="G9" s="3">
-        <f t="shared" ref="G9:G20" si="3">E9*F9</f>
+        <f t="shared" ref="G9:G20" si="4">E9*F9</f>
         <v>3.9899999999999998E-2</v>
       </c>
       <c r="H9" s="1" t="s">
@@ -1444,24 +1434,24 @@
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A10" s="34" t="s">
+      <c r="A10" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="38" t="s">
+      <c r="B10" s="32" t="s">
         <v>173</v>
       </c>
       <c r="D10">
         <v>1</v>
       </c>
       <c r="E10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F10" s="36">
+      <c r="F10" s="31">
         <v>1.3299999999999999E-2</v>
       </c>
       <c r="G10" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.9899999999999998E-2</v>
       </c>
       <c r="H10" s="1" t="s">
@@ -1478,24 +1468,24 @@
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A11" s="32" t="s">
+      <c r="A11" t="s">
         <v>139</v>
       </c>
-      <c r="B11" s="43" t="s">
+      <c r="B11" s="32" t="s">
         <v>174</v>
       </c>
       <c r="D11">
         <v>2</v>
       </c>
       <c r="E11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="F11" s="36">
+      <c r="F11" s="31">
         <v>0.18099999999999999</v>
       </c>
       <c r="G11" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.0859999999999999</v>
       </c>
       <c r="H11" s="1" t="s">
@@ -1528,22 +1518,22 @@
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
+      <c r="A12" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="38" t="s">
+      <c r="B12" s="32" t="s">
         <v>188</v>
       </c>
       <c r="D12">
         <v>8</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="40" t="s">
+      <c r="F12" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="41" t="s">
+      <c r="G12" s="35" t="s">
         <v>61</v>
       </c>
       <c r="H12" s="1" t="s">
@@ -1560,22 +1550,22 @@
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="38" t="s">
+      <c r="B13" s="32" t="s">
         <v>150</v>
       </c>
       <c r="D13">
         <v>1</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="F13" s="40" t="s">
+      <c r="F13" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="G13" s="41" t="s">
+      <c r="G13" s="35" t="s">
         <v>61</v>
       </c>
       <c r="H13" s="1" t="s">
@@ -1592,24 +1582,24 @@
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A14" s="34" t="s">
+      <c r="A14" t="s">
         <v>154</v>
       </c>
-      <c r="B14" s="38" t="s">
+      <c r="B14" s="32" t="s">
         <v>151</v>
       </c>
       <c r="D14">
         <v>2</v>
       </c>
       <c r="E14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="F14" s="36">
+      <c r="F14" s="31">
         <v>0.16</v>
       </c>
       <c r="G14" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.96</v>
       </c>
       <c r="H14" s="1" t="s">
@@ -1626,24 +1616,24 @@
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A15" s="34" t="s">
+      <c r="A15" t="s">
         <v>155</v>
       </c>
-      <c r="B15" s="38" t="s">
+      <c r="B15" s="32" t="s">
         <v>156</v>
       </c>
       <c r="D15">
         <v>2</v>
       </c>
       <c r="E15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="F15" s="36">
+      <c r="F15" s="31">
         <v>0.1</v>
       </c>
       <c r="G15" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.60000000000000009</v>
       </c>
       <c r="H15" s="1" t="s">
@@ -1660,24 +1650,24 @@
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A16" s="30" t="s">
+      <c r="A16" t="s">
         <v>164</v>
       </c>
-      <c r="B16" s="38" t="s">
+      <c r="B16" s="32" t="s">
         <v>14</v>
       </c>
       <c r="D16">
         <v>1</v>
       </c>
       <c r="E16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F16" s="36">
+      <c r="F16" s="31">
         <v>0.3</v>
       </c>
       <c r="G16" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0.89999999999999991</v>
       </c>
       <c r="H16" s="1" t="s">
@@ -1694,24 +1684,24 @@
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A17" s="30" t="s">
+      <c r="A17" t="s">
         <v>169</v>
       </c>
-      <c r="B17" s="42" t="s">
+      <c r="B17" s="36" t="s">
         <v>13</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F17" s="36">
+      <c r="F17" s="31">
         <v>0.64</v>
       </c>
       <c r="G17" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H17" s="1" t="s">
@@ -1728,22 +1718,22 @@
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A18" s="34" t="s">
+      <c r="A18" t="s">
         <v>175</v>
       </c>
-      <c r="B18" s="38" t="s">
+      <c r="B18" s="32" t="s">
         <v>186</v>
       </c>
       <c r="D18">
         <v>11</v>
       </c>
-      <c r="E18" s="39" t="s">
+      <c r="E18" s="33" t="s">
         <v>61</v>
       </c>
-      <c r="F18" s="40" t="s">
+      <c r="F18" s="34" t="s">
         <v>61</v>
       </c>
-      <c r="G18" s="41" t="s">
+      <c r="G18" s="35" t="s">
         <v>61</v>
       </c>
       <c r="H18" s="1" t="s">
@@ -1763,24 +1753,24 @@
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A19" s="34" t="s">
+      <c r="A19" t="s">
         <v>178</v>
       </c>
-      <c r="B19" s="38" t="s">
+      <c r="B19" s="32" t="s">
         <v>187</v>
       </c>
       <c r="D19">
         <v>2</v>
       </c>
       <c r="E19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="F19" s="36">
+      <c r="F19" s="31">
         <v>0.3</v>
       </c>
       <c r="G19" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1.7999999999999998</v>
       </c>
       <c r="H19" s="1" t="s">
@@ -1797,24 +1787,24 @@
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A20" s="34" t="s">
+      <c r="A20" t="s">
         <v>185</v>
       </c>
-      <c r="B20" s="38" t="s">
+      <c r="B20" s="32" t="s">
         <v>181</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="F20" s="36">
+      <c r="F20" s="31">
         <v>1.72</v>
       </c>
       <c r="G20" s="3">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5.16</v>
       </c>
       <c r="H20" s="1" t="s">
@@ -1832,525 +1822,525 @@
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N21" t="str">
-        <f t="shared" ref="N21:Q50" si="4">IF(ISNUMBER(SEARCH(N$1,$I21)),1,"")</f>
+        <f t="shared" ref="N21:Q50" si="5">IF(ISNUMBER(SEARCH(N$1,$I21)),1,"")</f>
         <v/>
       </c>
       <c r="O21" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P21" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q21" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q22" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N23" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O23" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P23" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q23" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N24" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O24" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P24" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q24" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N25" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O25" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P25" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q25" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q26" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N27" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O27" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P27" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q27" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="28" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q28" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N29" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O29" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P29" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q29" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="30" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N30" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O30" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P30" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q30" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N31" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O31" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P31" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q31" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="N32" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O32" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P32" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q32" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="33" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N33" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O33" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P33" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q33" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="34" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q34" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="35" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q35" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="36" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q36" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="37" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q37" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="38" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q38" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="39" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q39" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="40" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q40" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="41" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q41" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="42" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N42" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O42" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P42" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q42" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="43" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q43" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="44" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N44" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O44" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P44" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q44" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="45" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q45" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="46" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="Q46" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="47" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N47" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O47" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P47" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="48" spans="14:17" x14ac:dyDescent="0.2">
       <c r="N48" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O48" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P48" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="49" spans="14:16" x14ac:dyDescent="0.2">
       <c r="N49" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O49" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P49" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="50" spans="14:16" x14ac:dyDescent="0.2">
       <c r="N50" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="O50" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="P50" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>

</xml_diff>